<commit_message>
Envelope de voo por altitude adaptado do Envelope_main
- core/sim/envelope.zig: por altitude, V_min/V_max (P_d = P_r, grade +
  bisseção), V_e, V* = V_e·√n, V_cru e teto absoluto (bisseção em h).
  Método da planilha (opção de reproduzir o original exatamente) e método
  com a trimagem da aeronave completa.
- Tração como no original: T = g·(ρ/ρ0)·(T0 + p10·n + p01·V + ...), com x
  constante (n) no polinômio em comptime e T0 no lugar de p00.
- Mapa da planilha: AnguloCruzeiro, n, ρ0, C_Dp da asa/EH e K.
- Rotação de equilíbrio do motor por regula falsi (Illinois).
- GUI: gráfico altitude × velocidade, exportação .xlsx por tabela; casas
  decimais dos campos conforme o valor (tolerância 1e-5 virava 0).
- Testes: envelope = Envelope_main transcrito altitude por altitude.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Lfytn1estDGfcFH98sanGR
</commit_message>
<xml_diff>
--- a/data/aircraft/conventional.xlsx
+++ b/data/aircraft/conventional.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C134"/>
+  <dimension ref="A1:C142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2471,6 +2471,132 @@
       </c>
       <c r="C134" t="n">
         <v>15</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>performance</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>alpha_cruise</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>performance</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>load_factor</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>performance</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>rho0</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>1.225</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>performance</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>cdp_x</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>performance</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>cdp_wing</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>[0.0, 0.012]</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>performance</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>cdp_htail</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>[0.0, 0.012]</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>performance</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>K</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>performance</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>ceiling_min</t>
+        </is>
+      </c>
+      <c r="C142" t="n">
+        <v>500</v>
       </c>
     </row>
   </sheetData>
@@ -3300,7 +3426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV2"/>
+  <dimension ref="A1:AX2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3401,145 +3527,155 @@
       </c>
       <c r="T1" t="inlineStr">
         <is>
+          <t>thrust_poly.x_const</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>thrust_poly.y_const</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
           <t>thrust_poly.T0</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>thrust_poly.n</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>thrust_poly.source</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>motor.name</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>motor.Kv</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>motor.Rm</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>motor.B</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>motor.tauc</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>motor.Imax</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>motor.Jm</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>motor.mass</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>motor.source</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>propeller.name</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>propeller.D</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>propeller.pitch</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>propeller.Ip</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>propeller.mass</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>propeller.J</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>propeller.CT</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>propeller.CP</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>propeller.source</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>battery.name</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>battery.cells</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>battery.V_cell</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>battery.Rint</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>battery.capacity_mAh</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>battery.mass</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>battery.source</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>enabled</t>
         </is>
@@ -3621,105 +3757,111 @@
       <c r="U2" t="n">
         <v>0</v>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="V2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X2" t="inlineStr">
         <is>
           <t>""</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr">
+      <c r="Y2" t="inlineStr">
         <is>
           <t>Scorpion A-5025-310Kv</t>
         </is>
       </c>
-      <c r="X2" t="n">
+      <c r="Z2" t="n">
         <v>310</v>
       </c>
-      <c r="Y2" t="n">
+      <c r="AA2" t="n">
         <v>0.0204</v>
       </c>
-      <c r="Z2" t="n">
+      <c r="AB2" t="n">
         <v>3.24e-05</v>
       </c>
-      <c r="AA2" t="n">
+      <c r="AC2" t="n">
         <v>0.0155</v>
       </c>
-      <c r="AB2" t="n">
+      <c r="AD2" t="n">
         <v>80</v>
       </c>
-      <c r="AC2" t="n">
+      <c r="AE2" t="n">
         <v>0.0001</v>
       </c>
-      <c r="AD2" t="n">
+      <c r="AF2" t="n">
         <v>0.53</v>
       </c>
-      <c r="AE2" t="inlineStr">
+      <c r="AG2" t="inlineStr">
         <is>
           <t>dados do código original</t>
         </is>
       </c>
-      <c r="AF2" t="inlineStr">
+      <c r="AH2" t="inlineStr">
         <is>
           <t>APC 15x8E</t>
         </is>
       </c>
-      <c r="AG2" t="n">
+      <c r="AI2" t="n">
         <v>0.381</v>
       </c>
-      <c r="AH2" t="n">
+      <c r="AJ2" t="n">
         <v>0.2032</v>
       </c>
-      <c r="AI2" t="n">
+      <c r="AK2" t="n">
         <v>0.00054</v>
       </c>
-      <c r="AJ2" t="n">
+      <c r="AL2" t="n">
         <v>0.06</v>
       </c>
-      <c r="AK2" t="inlineStr">
+      <c r="AM2" t="inlineStr">
         <is>
           <t>[0.0, 0.0234, 0.0468, 0.0701, 0.0935, 0.1169, 0.1403, 0.1637, 0.1871, 0.2104, 0.2338, 0.2572, 0.2806, 0.304, 0.3274, 0.3507, 0.3741, 0.3975, 0.4209, 0.4443, 0.4676, 0.491, 0.5144, 0.5378, 0.5612, 0.5846, 0.6079, 0.6313, 0.6547, 0.6781]</t>
         </is>
       </c>
-      <c r="AL2" t="inlineStr">
+      <c r="AN2" t="inlineStr">
         <is>
           <t>[0.0896, 0.0883, 0.0869, 0.0853, 0.0836, 0.0818, 0.0799, 0.0778, 0.0756, 0.0732, 0.0706, 0.0679, 0.0651, 0.062, 0.0588, 0.0555, 0.052, 0.0484, 0.0446, 0.0407, 0.0368, 0.0327, 0.0286, 0.0245, 0.0203, 0.0162, 0.012, 0.0079, 0.0039, 0.0]</t>
         </is>
       </c>
-      <c r="AM2" t="inlineStr">
+      <c r="AO2" t="inlineStr">
         <is>
           <t>[0.0299, 0.0303, 0.0307, 0.031, 0.0314, 0.0316, 0.0319, 0.032, 0.0321, 0.0321, 0.032, 0.0317, 0.0314, 0.0309, 0.0304, 0.0296, 0.0288, 0.0278, 0.0266, 0.0253, 0.0239, 0.0224, 0.0207, 0.0189, 0.017, 0.015, 0.0129, 0.0108, 0.0085, 0.0062]</t>
         </is>
       </c>
-      <c r="AN2" t="inlineStr">
+      <c r="AP2" t="inlineStr">
         <is>
           <t>catálogo APC (6000 rpm)</t>
         </is>
       </c>
-      <c r="AO2" t="inlineStr">
+      <c r="AQ2" t="inlineStr">
         <is>
           <t>LiPo 6S 5000</t>
         </is>
       </c>
-      <c r="AP2" t="n">
+      <c r="AR2" t="n">
         <v>6</v>
       </c>
-      <c r="AQ2" t="n">
+      <c r="AS2" t="n">
         <v>3.7</v>
       </c>
-      <c r="AR2" t="n">
+      <c r="AT2" t="n">
         <v>0.035</v>
       </c>
-      <c r="AS2" t="n">
+      <c r="AU2" t="n">
         <v>5000</v>
       </c>
-      <c r="AT2" t="n">
+      <c r="AV2" t="n">
         <v>0.8</v>
       </c>
-      <c r="AU2" t="inlineStr">
+      <c r="AW2" t="inlineStr">
         <is>
           <t>dados do código original</t>
         </is>
       </c>
-      <c r="AV2" t="inlineStr">
+      <c r="AX2" t="inlineStr">
         <is>
           <t>true</t>
         </is>

</xml_diff>